<commit_message>
Deploying to gh-pages from  @ e11c32463dc3debf9126357d87988682de28fb5c 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_4-1-3.xlsx
+++ b/assets/excel/2026_4-1-3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0EC4A073-03C2-4EAB-89DA-F1E3358B5EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF6FCDF-1E86-4BC9-8282-51DF05217A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20052" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{95AE330F-3948-45C2-BEAB-3D17B9280608}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{95AE330F-3948-45C2-BEAB-3D17B9280608}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -382,7 +382,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -468,24 +468,8 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -541,12 +525,32 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -913,28 +917,28 @@
       <c r="L4" s="1"/>
     </row>
     <row r="6" spans="2:12" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="45" t="s">
+      <c r="D6" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="48" t="s">
+      <c r="E6" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="51" t="s">
+      <c r="F6" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="52"/>
+      <c r="G6" s="46"/>
     </row>
     <row r="7" spans="2:12" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="40"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="49"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="43"/>
       <c r="F7" s="8" t="s">
         <v>7</v>
       </c>
@@ -943,24 +947,24 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="40"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="46"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="53" t="s">
+      <c r="B8" s="34"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="51"/>
+      <c r="G8" s="45"/>
     </row>
     <row r="9" spans="2:12" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="41"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="47"/>
-      <c r="E9" s="54" t="s">
+      <c r="B9" s="35"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
     </row>
     <row r="10" spans="2:12" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="10">
@@ -5583,127 +5587,121 @@
       <c r="B216" s="30"/>
       <c r="D216" s="29"/>
     </row>
-    <row r="217" spans="2:16" s="22" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B217" s="56" t="s">
+    <row r="217" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B217" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="C217" s="56"/>
-      <c r="D217" s="56"/>
-      <c r="E217" s="56"/>
-      <c r="F217" s="56"/>
-      <c r="G217" s="56"/>
-      <c r="H217" s="56"/>
-      <c r="I217" s="56"/>
-      <c r="J217" s="56"/>
-      <c r="K217" s="56"/>
-      <c r="L217" s="56"/>
-      <c r="M217" s="56"/>
-      <c r="N217" s="56"/>
-      <c r="O217" s="56"/>
-      <c r="P217" s="56"/>
-    </row>
-    <row r="218" spans="2:16" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B218" s="31" t="s">
+      <c r="C217" s="50"/>
+      <c r="D217" s="50"/>
+      <c r="E217" s="50"/>
+      <c r="F217" s="50"/>
+      <c r="G217" s="50"/>
+      <c r="H217" s="50"/>
+      <c r="I217" s="50"/>
+      <c r="J217" s="50"/>
+      <c r="K217" s="50"/>
+      <c r="L217" s="50"/>
+      <c r="M217" s="50"/>
+      <c r="N217" s="50"/>
+      <c r="O217" s="50"/>
+      <c r="P217" s="50"/>
+    </row>
+    <row r="218" spans="2:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B218" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="C218" s="25"/>
-      <c r="D218" s="32"/>
-      <c r="E218" s="25"/>
-      <c r="F218" s="25"/>
-      <c r="G218" s="25"/>
-    </row>
-    <row r="219" spans="2:16" s="22" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B219" s="57" t="s">
+      <c r="C218" s="52"/>
+      <c r="D218" s="53"/>
+      <c r="E218" s="52"/>
+      <c r="F218" s="52"/>
+      <c r="G218" s="52"/>
+    </row>
+    <row r="219" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B219" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="C219" s="57"/>
-      <c r="D219" s="57"/>
-      <c r="E219" s="57"/>
-      <c r="F219" s="57"/>
-      <c r="G219" s="57"/>
-      <c r="H219" s="57"/>
-      <c r="I219" s="57"/>
-      <c r="J219" s="57"/>
-      <c r="K219" s="57"/>
-      <c r="L219" s="57"/>
-      <c r="M219" s="57"/>
-      <c r="N219" s="57"/>
-      <c r="O219" s="57"/>
-      <c r="P219" s="57"/>
-    </row>
-    <row r="220" spans="2:16" s="22" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B220" s="57" t="s">
+      <c r="C219" s="54"/>
+      <c r="D219" s="54"/>
+      <c r="E219" s="54"/>
+      <c r="F219" s="54"/>
+      <c r="G219" s="54"/>
+      <c r="H219" s="54"/>
+      <c r="I219" s="54"/>
+      <c r="J219" s="54"/>
+      <c r="K219" s="54"/>
+      <c r="L219" s="54"/>
+      <c r="M219" s="54"/>
+      <c r="N219" s="54"/>
+      <c r="O219" s="54"/>
+      <c r="P219" s="54"/>
+    </row>
+    <row r="220" spans="2:16" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B220" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="C220" s="57"/>
-      <c r="D220" s="57"/>
-      <c r="E220" s="57"/>
-      <c r="F220" s="57"/>
-      <c r="G220" s="57"/>
-      <c r="H220" s="57"/>
-      <c r="I220" s="57"/>
-      <c r="J220" s="57"/>
-      <c r="K220" s="57"/>
-      <c r="L220" s="57"/>
-      <c r="M220" s="57"/>
-      <c r="N220" s="57"/>
-      <c r="O220" s="57"/>
-      <c r="P220" s="57"/>
-    </row>
-    <row r="221" spans="2:16" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B221" s="33" t="s">
+      <c r="C220" s="54"/>
+      <c r="D220" s="54"/>
+      <c r="E220" s="54"/>
+      <c r="F220" s="54"/>
+      <c r="G220" s="54"/>
+      <c r="H220" s="54"/>
+      <c r="I220" s="54"/>
+      <c r="J220" s="54"/>
+      <c r="K220" s="54"/>
+      <c r="L220" s="54"/>
+      <c r="M220" s="54"/>
+      <c r="N220" s="54"/>
+      <c r="O220" s="54"/>
+      <c r="P220" s="54"/>
+    </row>
+    <row r="221" spans="2:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B221" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="C221" s="34"/>
-      <c r="D221" s="35"/>
-      <c r="E221" s="34"/>
-      <c r="F221" s="34"/>
-      <c r="G221" s="34"/>
-    </row>
-    <row r="222" spans="2:16" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B222" s="34"/>
-      <c r="C222" s="34"/>
-      <c r="D222" s="35"/>
-      <c r="E222" s="34"/>
-      <c r="F222" s="34"/>
-      <c r="G222" s="34"/>
-    </row>
-    <row r="223" spans="2:16" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B223" s="31" t="s">
+      <c r="C221" s="55"/>
+      <c r="D221" s="56"/>
+      <c r="E221" s="55"/>
+      <c r="F221" s="55"/>
+      <c r="G221" s="55"/>
+    </row>
+    <row r="222" spans="2:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B222" s="55"/>
+      <c r="C222" s="55"/>
+      <c r="D222" s="56"/>
+      <c r="E222" s="55"/>
+      <c r="F222" s="55"/>
+      <c r="G222" s="55"/>
+    </row>
+    <row r="223" spans="2:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B223" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="C223" s="36"/>
-      <c r="D223" s="37"/>
-      <c r="E223" s="28"/>
-      <c r="F223" s="28"/>
-      <c r="G223" s="28"/>
-    </row>
-    <row r="224" spans="2:16" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D224" s="29"/>
-    </row>
-    <row r="225" spans="2:4" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B225" s="31" t="s">
+      <c r="C223" s="57"/>
+      <c r="D223" s="58"/>
+      <c r="E223" s="59"/>
+      <c r="F223" s="59"/>
+      <c r="G223" s="59"/>
+    </row>
+    <row r="224" spans="2:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="225" spans="2:2" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B225" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="D225" s="29"/>
-    </row>
-    <row r="226" spans="2:4" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B226" s="31" t="s">
+    </row>
+    <row r="226" spans="2:2" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B226" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="D226" s="29"/>
-    </row>
-    <row r="227" spans="2:4" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B227" s="31" t="s">
+    </row>
+    <row r="227" spans="2:2" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B227" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="D227" s="29"/>
-    </row>
-    <row r="228" spans="2:4" s="22" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B228" s="38" t="s">
+    </row>
+    <row r="228" spans="2:2" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B228" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="D228" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -5719,8 +5717,8 @@
     <mergeCell ref="E9:G9"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B228" r:id="rId1" xr:uid="{0178E4F1-5847-4B81-ADBB-EFDE3517656C}"/>
-    <hyperlink ref="B221" r:id="rId2" xr:uid="{4B446814-EB3D-4088-8F8C-638339A7752C}"/>
+    <hyperlink ref="B228" r:id="rId1" xr:uid="{6FAAC617-D352-43BC-89B5-03CBC39EC40B}"/>
+    <hyperlink ref="B221" r:id="rId2" xr:uid="{61792E8D-BD81-4DE6-BE17-43CFD54D934C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>